<commit_message>
[Modify][MOS_EXCEL_THI] fix function and question
</commit_message>
<xml_diff>
--- a/Data/Excel_Thi/data/5.xlsx
+++ b/Data/Excel_Thi/data/5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\MOS360\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell7390\Desktop\File đề test\TEST EXCEL_11P\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{545D5BB3-49CB-4F02-A4D4-A2FBEA9D0445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6BDFA4-1DE2-4259-A0B7-D9ABE0EE326D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-30" windowWidth="28920" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quote" sheetId="1" r:id="rId1"/>
@@ -24,21 +24,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="61">
   <si>
     <t>VanArsdel, Ltd</t>
   </si>
@@ -218,6 +209,9 @@
   </si>
   <si>
     <t>March</t>
+  </si>
+  <si>
+    <t>Prices</t>
   </si>
 </sst>
 </file>
@@ -231,14 +225,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -246,7 +240,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -254,7 +248,7 @@
       <b/>
       <sz val="16"/>
       <color theme="0"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -263,7 +257,7 @@
       <b/>
       <sz val="12"/>
       <color theme="5"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -272,14 +266,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2410,20 +2404,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:H33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
     <col min="2" max="2" width="4" customWidth="1"/>
-    <col min="3" max="3" width="6.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" customWidth="1"/>
-    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.25" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:8" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2432,7 +2426,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="2:8" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="4"/>
       <c r="C3" s="30" t="s">
         <v>0</v>
@@ -2443,11 +2437,11 @@
       <c r="G3" s="30"/>
       <c r="H3" s="5"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="4"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="4"/>
       <c r="C5" s="31" t="s">
         <v>1</v>
@@ -2458,18 +2452,18 @@
       <c r="G5" s="31"/>
       <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="4"/>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" spans="2:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="4"/>
       <c r="D7" s="22" t="s">
         <v>2</v>
       </c>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" spans="2:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="D8" s="22" t="s">
         <v>3</v>
@@ -2478,7 +2472,7 @@
       <c r="F8" s="17"/>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" spans="2:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="4"/>
       <c r="D9" s="22" t="s">
         <v>4</v>
@@ -2487,7 +2481,7 @@
       <c r="F9" s="17"/>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" spans="2:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
       <c r="D10" s="22" t="s">
         <v>5</v>
@@ -2496,13 +2490,13 @@
       <c r="F10" s="17"/>
       <c r="H10" s="5"/>
     </row>
-    <row r="11" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="4"/>
       <c r="E11" s="28"/>
       <c r="F11" s="29"/>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="4"/>
       <c r="C12" s="13" t="s">
         <v>7</v>
@@ -2515,7 +2509,7 @@
       </c>
       <c r="H12" s="5"/>
     </row>
-    <row r="13" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="4"/>
       <c r="C13" s="18" t="s">
         <v>9</v>
@@ -2535,7 +2529,7 @@
       </c>
       <c r="H13" s="5"/>
     </row>
-    <row r="14" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="4"/>
       <c r="C14" s="18" t="s">
         <v>10</v>
@@ -2555,7 +2549,7 @@
       </c>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="4"/>
       <c r="C15" s="18" t="s">
         <v>11</v>
@@ -2575,7 +2569,7 @@
       </c>
       <c r="H15" s="5"/>
     </row>
-    <row r="16" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="4"/>
       <c r="C16" s="20"/>
       <c r="D16" s="19"/>
@@ -2588,7 +2582,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="5"/>
     </row>
-    <row r="17" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="4"/>
       <c r="C17" s="20"/>
       <c r="D17" s="19"/>
@@ -2597,7 +2591,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="5"/>
     </row>
-    <row r="18" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="4"/>
       <c r="C18" s="20"/>
       <c r="D18" s="19"/>
@@ -2606,7 +2600,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="5"/>
     </row>
-    <row r="19" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="4"/>
       <c r="C19" s="20"/>
       <c r="D19" s="19"/>
@@ -2615,7 +2609,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="4"/>
       <c r="C20" s="20"/>
       <c r="D20" s="19"/>
@@ -2624,7 +2618,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="5"/>
     </row>
-    <row r="21" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="4"/>
       <c r="C21" s="20"/>
       <c r="D21" s="19"/>
@@ -2633,7 +2627,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="5"/>
     </row>
-    <row r="22" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="4"/>
       <c r="C22" s="20"/>
       <c r="D22" s="19"/>
@@ -2642,7 +2636,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="5"/>
     </row>
-    <row r="23" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="4"/>
       <c r="C23" s="20"/>
       <c r="D23" s="19"/>
@@ -2651,7 +2645,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="5"/>
     </row>
-    <row r="24" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="4"/>
       <c r="C24" s="20"/>
       <c r="D24" s="19"/>
@@ -2660,7 +2654,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="5"/>
     </row>
-    <row r="25" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="4"/>
       <c r="C25" s="20"/>
       <c r="D25" s="19"/>
@@ -2669,7 +2663,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="5"/>
     </row>
-    <row r="26" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="4"/>
       <c r="C26" s="20"/>
       <c r="D26" s="19"/>
@@ -2678,7 +2672,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="5"/>
     </row>
-    <row r="27" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="4"/>
       <c r="C27" s="20"/>
       <c r="D27" s="19"/>
@@ -2687,7 +2681,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="4"/>
       <c r="E28" s="20"/>
       <c r="F28" s="21"/>
@@ -2697,7 +2691,7 @@
       </c>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B29" s="4"/>
       <c r="F29" s="9" t="s">
         <v>17</v>
@@ -2707,7 +2701,7 @@
       </c>
       <c r="H29" s="5"/>
     </row>
-    <row r="30" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="4"/>
       <c r="F30" s="9" t="s">
         <v>18</v>
@@ -2718,7 +2712,7 @@
       </c>
       <c r="H30" s="5"/>
     </row>
-    <row r="31" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -2728,11 +2722,11 @@
       <c r="G31" s="7"/>
       <c r="H31" s="8"/>
     </row>
-    <row r="32" spans="2:8" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
     </row>
-    <row r="33" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="33" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="E11:F11"/>
@@ -2747,21 +2741,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="4" max="4" width="9.375" customWidth="1"/>
-    <col min="5" max="5" width="14.625" customWidth="1"/>
-    <col min="6" max="6" width="15.75" customWidth="1"/>
-    <col min="7" max="7" width="16.5" customWidth="1"/>
-    <col min="8" max="8" width="10.25" customWidth="1"/>
-    <col min="9" max="9" width="10.625" customWidth="1"/>
-    <col min="10" max="10" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.75" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="10.21875" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" customWidth="1"/>
+    <col min="10" max="10" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
       <c r="J1" s="24" t="s">
         <v>30</v>
       </c>
@@ -2769,7 +2766,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="J2" s="23">
         <v>1</v>
       </c>
@@ -2777,8 +2774,8 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>20</v>
       </c>
@@ -2813,7 +2810,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>CONCATENATE(B5, " ",C5," (Unisex)")</f>
         <v>Hoodie Black (Unisex)</v>
@@ -2847,7 +2844,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f t="shared" ref="A6:A25" si="0">CONCATENATE(B6, " ",C6," (Unisex)")</f>
         <v>Hoodie Blue (Unisex)</v>
@@ -2881,7 +2878,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Hoodie Green (Unisex)</v>
@@ -2915,7 +2912,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>Hoodie Orange (Unisex)</v>
@@ -2949,7 +2946,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>Hoodie Purple (Unisex)</v>
@@ -2983,7 +2980,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>Hoodie Red (Unisex)</v>
@@ -3017,7 +3014,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>Hoodie White (Unisex)</v>
@@ -3051,7 +3048,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Black (Unisex)</v>
@@ -3085,7 +3082,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Blue (Unisex)</v>
@@ -3119,7 +3116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Green (Unisex)</v>
@@ -3153,7 +3150,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Orange (Unisex)</v>
@@ -3187,7 +3184,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Purple (Unisex)</v>
@@ -3221,7 +3218,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt Red (Unisex)</v>
@@ -3255,7 +3252,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>Sweatshirt White (Unisex)</v>
@@ -3289,7 +3286,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Black (Unisex)</v>
@@ -3323,7 +3320,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Blue (Unisex)</v>
@@ -3357,7 +3354,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Green (Unisex)</v>
@@ -3391,7 +3388,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Orange (Unisex)</v>
@@ -3425,7 +3422,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Purple (Unisex)</v>
@@ -3459,7 +3456,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt Red (Unisex)</v>
@@ -3493,7 +3490,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>T-Shirt White (Unisex)</v>
@@ -3539,7 +3536,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3549,16 +3546,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E38"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.125" customWidth="1"/>
-    <col min="3" max="3" width="12.125" customWidth="1"/>
-    <col min="4" max="4" width="18.125" customWidth="1"/>
-    <col min="5" max="5" width="12.375" customWidth="1"/>
+    <col min="1" max="1" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -3575,7 +3572,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -3592,7 +3589,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -3609,7 +3606,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -3626,7 +3623,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -3643,7 +3640,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -3660,7 +3657,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -3677,7 +3674,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>52</v>
       </c>
@@ -3694,7 +3691,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -3711,7 +3708,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -3728,7 +3725,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -3745,7 +3742,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -3762,7 +3759,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>51</v>
       </c>
@@ -3779,7 +3776,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -3796,7 +3793,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -3813,7 +3810,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -3830,7 +3827,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -3847,7 +3844,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -3864,7 +3861,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>56</v>
       </c>
@@ -3881,7 +3878,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>50</v>
       </c>
@@ -3898,7 +3895,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -3915,7 +3912,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -3932,7 +3929,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>47</v>
       </c>
@@ -3949,7 +3946,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -3966,7 +3963,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>56</v>
       </c>
@@ -3983,7 +3980,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>47</v>
       </c>
@@ -4000,7 +3997,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -4017,7 +4014,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>48</v>
       </c>
@@ -4034,7 +4031,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>55</v>
       </c>
@@ -4051,7 +4048,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -4068,7 +4065,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>51</v>
       </c>
@@ -4085,7 +4082,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>53</v>
       </c>
@@ -4102,7 +4099,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>47</v>
       </c>
@@ -4119,7 +4116,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -4136,7 +4133,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>48</v>
       </c>
@@ -4153,7 +4150,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -4170,7 +4167,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>56</v>
       </c>
@@ -4187,7 +4184,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B38" s="27"/>
     </row>
   </sheetData>
@@ -4202,7 +4199,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>